<commit_message>
feat(F-NAR-019): ATOM-EMO.LEX.001-07 Mila et la fraise tiède
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-EMO.LEX.001-07.xlsx
+++ b/stories/arbres/ATOM-EMO.LEX.001-07.xlsx
@@ -671,7 +671,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>jardin, fraisiers, fin de journée</t>
+          <t>jardin, fraisiers, fin de journée, arrosoir, seau, brouette, terre, feuilles, fer</t>
         </is>
       </c>
     </row>
@@ -841,7 +841,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>L'arrosoir goutte. Mila trouve une fraise tiède. Elle dit sa joie. Elle la partage avec maman et papa.</t>
+          <t>Une goutte reste au bec de l'arrosoir. Sur le fer, un éclat de brouette luit. Mila veut la fraise tiède, maintenant. Elle tire trop vite. La fraise est trop molle. Jus sur les doigts. Sourire parti. Papa s'accroupit. Elle tend, dit : je suis contente. Merci vécu. Deuxième ruse : un oiseau, le jus, la fraise trop molle. Elle refuse de foncer. Un éclat de brouette tient sur le fer.</t>
         </is>
       </c>
     </row>
@@ -1184,17 +1184,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>L'arrosoir goutte encore dans l'herbe. La terre sent le chaud. Un seau de bois est encore mouillé. Des tomates vertes pendent plus loin. Le soleil est bas, tout orange. Une coccinelle marche sur une feuille. Les feuilles des fraisiers sont un peu poussiéreuses. Maman pose l'arrosoir près du bac. Papa arrive du fond du jardin, les mains pleines de terre. Mila, tu veux chercher sous les feuilles ? Oui. Les fraises se cachent. On marche entre les rangs, tout doux. En ce moment, Mila s'accroupit. La terre est tiède sous ses genoux. Un caillou roule sous sa chaussure. Une feuille sent le vert. Sous la feuille, une fraise rouge. Elle est petite. Elle est tiède. Je l'ai ! Tu la cueilles tout doucement. Mila la détache. La queue reste verte. Parce qu'elle a trouvé la fraise, ses joues deviennent chaudes. Son ventre est léger. Un sourire arrive. Je suis contente. C'est de la joie. Tu as nommé ta joie. Bravo, Mila. On peut partager ? Oui. On partage. Mila tend la fraise. Maman croque un bout. Papa croque un bout. Mila croque le dernier bout. C'est sucré. C'est un peu chaud du soleil. Merci. Tu nous invites. Je suis contente. Tu as encore de la joie ? Oui, maman. L'arrosoir fait encore une goutte. La goutte tombe dans l'herbe.</t>
+          <t>Une goutte reste au bec de l'arrosoir. Elle pend, papa. Tu la vois, la goutte ? Oui, elle brille. La terre du rang sent le soleil. Ça sent la terre, maman. Tu la sens, la terre chaude ? Oui, maman. Le seau de bois est mouillé, près des pieds. Il sent l'eau. Il a bu le rang. Maman pose l'arrosoir contre la brouette. Le fer de la brouette est tiède. Il est chaud ! Le soleil l'a touché. Sur le fer, un éclat de brouette luit. Il brille, maman. Tu le vois, le petit point ? Oui, un petit point. Papa a de la terre aux mains. Les feuilles des fraisiers sont poussiéreuses. Elles cachent des rouges. Tu veux chercher, Mila ? Oui, maintenant ! En ce moment, Mila s'accroupit. La terre est tiède sous ses genoux. Elle chauffe. Tes genoux sont bien ? Oui, papa. Une feuille sent le vert, tout près. Tu la lèves, Mila ? Oui. Sous la feuille, une fraise rouge. Elle est petite ! Elle est tiède, sous la feuille. Je la prends, maintenant ! Mila tire trop vite, trop fort. La fraise est trop molle. Oh. Le jus rougit ses doigts. La fraise glisse, presque. Elle glisse ! Le sourire de Mila disparaît. Dans sa poitrine, ça se bouscule. L'envie et la peur se heurtent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu vois tes doigts, Mila ? Ils sont rouges. La fraise est molle, Mila ? Un peu, maman. L'éclat de brouette tremble, puis tient. Mila referme les doigts, sans serrer. Elle est chaude. Tu la tiens ? Oui, papa. Mila veut croquer, tout de suite. Je la mange, maintenant ! Les mots se bousculent dans sa bouche. Elle avance la fraise vers sa bouche. Puis elle s'arrête. Elle regarde papa, puis maman. Pour vous aussi. Ses joues sont chaudes. Elle tend la fraise, sans bousculer. Je suis contente. Elle sent le soleil. On la goûte où ?</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>L'arrosoir goutte encore dans l'herbe. La terre sent le chaud. Un seau de bois est encore mouillé. Des tomates vertes pendent plus loin. Le soleil est bas, tout orange. Une coccinelle marche sur une feuille. Les feuilles des fraisiers sont un peu poussiéreuses. Maman pose l'arrosoir près du bac. Papa arrive du fond du jardin, les mains pleines de terre. Mila, tu veux chercher sous les feuilles ? Oui. Les fraises se cachent. On marche entre les rangs, tout doux. En ce moment, Mila s'accroupit. La terre est tiède sous ses genoux. Un caillou roule sous sa chaussure. Une feuille sent le vert. Sous la feuille, une fraise rouge. Elle est petite. Elle est tiède. Je l'ai ! Tu la cueilles tout doucement. Mila la détache. La queue reste verte. Parce qu'elle a trouvé la fraise, ses joues deviennent chaudes. Son ventre est léger. Un sourire arrive. Je suis contente. C'est de la joie. Tu as nommé ta joie. Bravo, Mila. On peut partager ? Oui. On partage. Mila tend la fraise. Maman croque un bout. Papa croque un bout. Mila croque le dernier bout. C'est sucré. C'est un peu chaud du soleil. Merci. Tu nous invites. Je suis contente. Tu as encore de la joie ? Oui, maman. L'arrosoir fait encore une goutte. La goutte tombe dans l'herbe.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Une goutte reste au bec de l'arrosoir. Elle pend, papa. Tu la vois, la goutte ? Oui, elle brille. La terre du rang sent le soleil. Ça sent la terre, maman. Tu la sens, la terre chaude ? Oui, maman. Le seau de bois est mouillé, près des pieds. Il sent l'eau. Il a bu le rang. Maman pose l'arrosoir contre la brouette. Le fer de la brouette est tiède. Il est chaud ! Le soleil l'a touché. Sur le fer, un &lt;emphasis level="moderate"&gt;éclat de brouette&lt;/emphasis&gt; luit. Il brille, maman. Tu le vois, le petit point ? Oui, un petit point. Papa a de la terre aux mains. Les feuilles des fraisiers sont poussiéreuses. Elles cachent des rouges. Tu veux chercher, Mila ? Oui, maintenant ! En ce moment, Mila s'accroupit. La terre est tiède sous ses genoux. Elle chauffe. Tes genoux sont bien ? Oui, papa. Une feuille sent le vert, tout près. Tu la lèves, Mila ? Oui. Sous la feuille, une fraise rouge. Elle est petite ! Elle est tiède, sous la feuille. Je la prends, maintenant ! Mila tire trop vite, trop fort. La fraise est trop molle. Oh. Le jus rougit ses doigts. La fraise glisse, presque. Elle glisse ! Le sourire de Mila disparaît. Dans sa poitrine, ça se bouscule. L'envie et la peur se heurtent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu vois tes doigts, Mila ? Ils sont rouges. La fraise est molle, Mila ? Un peu, maman. L'éclat de brouette tremble, puis tient. Mila referme les doigts, sans serrer. Elle est chaude. Tu la tiens ? Oui, papa. Mila veut croquer, tout de suite. Je la mange, maintenant ! Les mots se bousculent dans sa bouche. Elle avance la fraise vers sa bouche. Puis elle s'arrête. Elle regarde papa, puis maman. Pour vous aussi. Ses joues sont chaudes. Elle tend la fraise, sans bousculer. Je suis contente. Elle sent le soleil. On la goûte où ?&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Émeline est dans le jardin avec maman. Les feuilles sentent le vert. Émeline trouve une fraise rouge. Elle est tiède. Parce qu'elle a trouvé la fraise, Émeline sent ses joues chaudes. Son ventre est léger. Un sourire arrive. Émeline dit : je suis &lt;emphasis&gt;content&lt;/emphasis&gt;e. Papa arrive près du potager. Papa dit : c'est de la joie. Émeline tend la fraise. Elle dit : on peut partager. Maman croque un bout. Papa croque un bout. Ils sourient ensemble. Émeline dit encore : je suis contente. La joie est là, près des fraisiers. [pause]</t>
+          <t>Une goutte reste au bec de l'arrosoir. Elle pend, papa. Tu la vois, la goutte ? Oui, elle brille. La terre du rang sent le soleil. Ça sent la terre, maman. Tu la sens, la terre chaude ? Oui, maman. Le seau de bois est mouillé, près des pieds. Il sent l'eau. Il a bu le rang. Maman pose l'arrosoir contre la brouette. Le fer de la brouette est tiède. Il est chaud ! Le soleil l'a touché. Sur le fer, un &lt;emphasis&gt;éclat de brouette&lt;/emphasis&gt; luit. Il brille, maman. Tu le vois, le petit point ? Oui, un petit point. Papa a de la terre aux mains. Les feuilles des fraisiers sont poussiéreuses. Elles cachent des rouges. Tu veux chercher, Mila ? Oui, maintenant ! En ce moment, Mila s'accroupit. La terre est tiède sous ses genoux. Elle chauffe. Tes genoux sont bien ? Oui, papa. Une feuille sent le vert, tout près. Tu la lèves, Mila ? Oui. Sous la feuille, une fraise rouge. Elle est petite ! Elle est tiède, sous la feuille. Je la prends, maintenant ! Mila tire trop vite, trop fort. La fraise est trop molle. Oh. Le jus rougit ses doigts. La fraise glisse, presque. Elle glisse ! Le sourire de Mila disparaît. Dans sa poitrine, ça se bouscule. L'envie et la peur se heurtent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu vois tes doigts, Mila ? Ils sont rouges. La fraise est molle, Mila ? Un peu, maman. L'éclat de brouette tremble, puis tient. Mila referme les doigts, sans serrer. Elle est chaude. Tu la tiens ? Oui, papa. Mila veut croquer, tout de suite. Je la mange, maintenant ! Les mots se bousculent dans sa bouche. Elle avance la fraise vers sa bouche. Puis elle s'arrête. Elle regarde papa, puis maman. Pour vous aussi. Ses joues sont chaudes. Elle tend la fraise, sans bousculer. Je suis contente. Elle sent le soleil. On la goûte où ? [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>132</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1249,10 +1249,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.18</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1275,30 +1275,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>content</t>
+          <t>éclat de brouette</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1307,10 +1307,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1321,48 +1321,81 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis inquiétude; intensite=2; destinataire=enfant; sous_texte=elle_veut_la_fraise_tiède_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|L'arrosoir goutte encore dans l'herbe.
-narrateur|La terre sent le chaud.
-narrateur|Un seau de bois est encore mouillé.
-narrateur|Des tomates vertes pendent plus loin.
-narrateur|Le soleil est bas, tout orange.
-narrateur|Une coccinelle marche sur une feuille.
-narrateur|Les feuilles des fraisiers sont un peu poussiéreuses.
-narrateur|Maman pose l'arrosoir près du bac.
-narrateur|Papa arrive du fond du jardin, les mains pleines de terre.
-maman|Mila, tu veux chercher sous les feuilles ?
-enfant-f|Oui. Les fraises se cachent.
-papa|On marche entre les rangs, tout doux.
+          <t>narrateur|Une goutte reste au bec de l'arrosoir.
+enfant-f|Elle pend, papa.
+papa|Tu la vois, la goutte ?
+enfant-f|Oui, elle brille.
+narrateur|La terre du rang sent le soleil.
+enfant-f|Ça sent la terre, maman.
+maman|Tu la sens, la terre chaude ?
+enfant-f|Oui, maman.
+narrateur|Le seau de bois est mouillé, près des pieds.
+enfant-f|Il sent l'eau.
+papa|Il a bu le rang.
+narrateur|Maman pose l'arrosoir contre la brouette.
+narrateur|Le fer de la brouette est tiède.
+enfant-f|Il est chaud !
+maman|Le soleil l'a touché.
+narrateur|Sur le fer, un éclat de brouette luit.
+enfant-f|Il brille, maman.
+maman|Tu le vois, le petit point ?
+enfant-f|Oui, un petit point.
+narrateur|Papa a de la terre aux mains.
+narrateur|Les feuilles des fraisiers sont poussiéreuses.
+enfant-f|Elles cachent des rouges.
+maman|Tu veux chercher, Mila ?
+enfant-f|Oui, maintenant !
 narrateur|En ce moment, Mila s'accroupit.
 narrateur|La terre est tiède sous ses genoux.
-narrateur|Un caillou roule sous sa chaussure.
-narrateur|Une feuille sent le vert.
+enfant-f|Elle chauffe.
+papa|Tes genoux sont bien ?
+enfant-f|Oui, papa.
+narrateur|Une feuille sent le vert, tout près.
+maman|Tu la lèves, Mila ?
+enfant-f|Oui.
 narrateur|Sous la feuille, une fraise rouge.
-narrateur|Elle est petite. Elle est tiède.
-enfant-f|Je l'ai !
-maman|Tu la cueilles tout doucement.
-narrateur|Mila la détache. La queue reste verte.
-narrateur|Parce qu'elle a trouvé la fraise, ses joues deviennent chaudes.
-narrateur|Son ventre est léger.
-narrateur|Un sourire arrive.
+enfant-f|Elle est petite !
+narrateur|Elle est tiède, sous la feuille.
+enfant-f|Je la prends, maintenant !
+narrateur|Mila tire trop vite, trop fort.
+narrateur|La fraise est trop molle.
+enfant-f|Oh.
+narrateur|Le jus rougit ses doigts.
+narrateur|La fraise glisse, presque.
+enfant-f|Elle glisse !
+narrateur|Le sourire de Mila disparaît.
+narrateur|Dans sa poitrine, ça se bouscule.
+narrateur|L'envie et la peur se heurtent.
+narrateur|Ses épaules tombent un peu.
+narrateur|Papa s'accroupit à la même hauteur.
+papa|Tu vois tes doigts, Mila ?
+enfant-f|Ils sont rouges.
+maman|La fraise est molle, Mila ?
+enfant-f|Un peu, maman.
+narrateur|L'éclat de brouette tremble, puis tient.
+narrateur|Mila referme les doigts, sans serrer.
+enfant-f|Elle est chaude.
+papa|Tu la tiens ?
+enfant-f|Oui, papa.
+narrateur|Mila veut croquer, tout de suite.
+enfant-f|Je la mange, maintenant !
+narrateur|Les mots se bousculent dans sa bouche.
+narrateur|Elle avance la fraise vers sa bouche.
+narrateur|Puis elle s'arrête.
+narrateur|Elle regarde papa, puis maman.
+enfant-f|Pour vous aussi.
+narrateur|Ses joues sont chaudes.
+narrateur|Elle tend la fraise, sans bousculer.
 enfant-f|Je suis contente.
-papa|C'est de la joie.
-maman|Tu as nommé ta joie. Bravo, Mila.
-enfant-f|On peut partager ?
-maman|Oui. On partage.
-narrateur|Mila tend la fraise.
-narrateur|Maman croque un bout. Papa croque un bout.
-narrateur|Mila croque le dernier bout.
-narrateur|C'est sucré. C'est un peu chaud du soleil.
-papa|Merci. Tu nous invites.
-enfant-f|Je suis contente.
-maman|Tu as encore de la joie ?
-enfant-f|Oui, maman.
-narrateur|L'arrosoir fait encore une goutte.
-narrateur|La goutte tombe dans l'herbe.</t>
+maman|Elle sent le soleil.
+papa|On la goûte où ?</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
@@ -1399,12 +1432,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Mila sourit. Que dit-elle ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;&lt;emphasis level="moderate"&gt;Mila&lt;/emphasis&gt; sourit. Que dit-elle ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Émeline sourit. Que dit-elle ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;&lt;emphasis&gt;Mila&lt;/emphasis&gt; sourit. Que dit-elle ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1429,7 +1462,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>Émeline sent de la joie. Que dit-elle ?</t>
+          <t>Mila sent de la joie. Que dit-elle ?</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr"/>
@@ -1467,7 +1500,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1478,7 +1511,7 @@
         <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.3</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1493,34 +1526,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>Mila</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1535,22 +1572,23 @@
         <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=mila_sourit_que_dit_elle; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
         <is>
-          <t>narrateur|Mila sourit. Que dit-elle ?</t>
+          <t>narrateur|Mila sourit.
+narrateur|Que dit-elle ?</t>
         </is>
       </c>
     </row>
@@ -1577,17 +1615,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Mila a encore un peu de rouge au doigt. C'est de la joie. Oui. Tu es contente. Tu as partagé ta fraise. Tu as fini ton petit bout ? Oui. Mila essuie ses doigts sur l'herbe. Les fraisiers restent tout bas.</t>
+          <t>Maman se baisse vers la fraise. Papa reste à la même hauteur. Un bout pour maman. Tout petit, Mila ? Oui, elle est molle. Mila avance trop vite vers maman. Le jus coule sur le pouce. Il coule ! Les mots se bousculent dans sa bouche. Vite, le bout ! Mila avance les mains, trop vite. Puis elle s'arrête. Mila refuse de foncer. Elle referme la bouche. Personne ne parle. Elle observe la fraise, un instant. Elle écoute le jardin. Tu restes un peu, Mila ? Oui, papa. Merci, Mila. Mila tend un bout, sans serrer. Maman croque un tout petit bout. Elle est tiède, sous la langue. Comme le soleil. Un bout pour moi ? Oui, papa. Papa croque, sans serrer. Il reste le mien. Tes doigts sont rouges, Mila ? Un peu, maman. Le ventre de Mila se desserre. Les épaules se relèvent un peu. On reste près de la brouette ? Oui. Mila tient le dernier bout à deux mains. Je ne serre pas.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Mila a encore un peu de rouge au doigt. C'est de la joie. Oui. Tu es contente. Tu as partagé ta fraise. Tu as fini ton petit bout ? Oui. Mila essuie ses doigts sur l'herbe. Les fraisiers restent tout bas.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Maman se baisse vers la &lt;emphasis level="moderate"&gt;fraise&lt;/emphasis&gt;. Papa reste à la même hauteur. Un bout pour maman. Tout petit, Mila ? Oui, elle est molle. Mila avance trop vite vers maman. Le jus coule sur le pouce. Il coule ! Les mots se bousculent dans sa bouche. Vite, le bout ! Mila avance les mains, trop vite. Puis elle s'arrête. Mila refuse de foncer. Elle referme la bouche. Personne ne parle. Elle observe la fraise, un instant. Elle écoute le jardin. Tu restes un peu, Mila ? Oui, papa. Merci, Mila. Mila tend un bout, sans serrer. Maman croque un tout petit bout. Elle est tiède, sous la langue. Comme le soleil. Un bout pour moi ? Oui, papa. Papa croque, sans serrer. Il reste le mien. Tes doigts sont rouges, Mila ? Un peu, maman. Le ventre de Mila se desserre. Les épaules se relèvent un peu. On reste près de la brouette ? Oui. Mila tient le dernier bout à deux mains. Je ne serre pas.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Émeline a nommé sa joie. Elle a partagé avec papa et maman. Être &lt;emphasis&gt;content&lt;/emphasis&gt;, c'est bien. [pause]</t>
+          <t>Maman se baisse vers la &lt;emphasis&gt;fraise&lt;/emphasis&gt;. Papa reste à la même hauteur. Un bout pour maman. Tout petit, Mila ? Oui, elle est molle. Mila avance trop vite vers maman. Le jus coule sur le pouce. Il coule ! Les mots se bousculent dans sa bouche. Vite, le bout ! Mila avance les mains, trop vite. Puis elle s'arrête. Mila refuse de foncer. Elle referme la bouche. Personne ne parle. Elle observe la fraise, un instant. Elle écoute le jardin. Tu restes un peu, Mila ? Oui, papa. Merci, Mila. Mila tend un bout, sans serrer. Maman croque un tout petit bout. Elle est tiède, sous la langue. Comme le soleil. Un bout pour moi ? Oui, papa. Papa croque, sans serrer. Il reste le mien. Tes doigts sont rouges, Mila ? Un peu, maman. Le ventre de Mila se desserre. Les épaules se relèvent un peu. On reste près de la brouette ? Oui. Mila tient le dernier bout à deux mains. Je ne serre pas. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1634,7 +1672,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>132</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1642,10 +1680,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.18</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1668,30 +1706,30 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>content</t>
+          <t>fraise</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1700,10 +1738,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1716,19 +1754,47 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=retenue puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=elle_tend_sans_foncer_ils_goûtent; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Mila a encore un peu de rouge au doigt.
-enfant-f|C'est de la joie.
-maman|Oui. Tu es contente.
-maman|Tu as partagé ta fraise.
-papa|Tu as fini ton petit bout ?
+          <t>narrateur|Maman se baisse vers la fraise.
+narrateur|Papa reste à la même hauteur.
+enfant-f|Un bout pour maman.
+maman|Tout petit, Mila ?
+enfant-f|Oui, elle est molle.
+narrateur|Mila avance trop vite vers maman.
+narrateur|Le jus coule sur le pouce.
+enfant-f|Il coule !
+narrateur|Les mots se bousculent dans sa bouche.
+enfant-f|Vite, le bout !
+narrateur|Mila avance les mains, trop vite.
+narrateur|Puis elle s'arrête.
+narrateur|Mila refuse de foncer.
+narrateur|Elle referme la bouche.
+narrateur|Personne ne parle.
+narrateur|Elle observe la fraise, un instant.
+narrateur|Elle écoute le jardin.
+papa|Tu restes un peu, Mila ?
+enfant-f|Oui, papa.
+papa|Merci, Mila.
+narrateur|Mila tend un bout, sans serrer.
+narrateur|Maman croque un tout petit bout.
+maman|Elle est tiède, sous la langue.
+enfant-f|Comme le soleil.
+papa|Un bout pour moi ?
+enfant-f|Oui, papa.
+narrateur|Papa croque, sans serrer.
+enfant-f|Il reste le mien.
+maman|Tes doigts sont rouges, Mila ?
+enfant-f|Un peu, maman.
+narrateur|Le ventre de Mila se desserre.
+narrateur|Les épaules se relèvent un peu.
+papa|On reste près de la brouette ?
 enfant-f|Oui.
-narrateur|Mila essuie ses doigts sur l'herbe.
-narrateur|Les fraisiers restent tout bas.</t>
+narrateur|Mila tient le dernier bout à deux mains.
+enfant-f|Je ne serre pas.</t>
         </is>
       </c>
     </row>
@@ -1755,17 +1821,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Mila se relève. La terre est tiède. On rentre l'arrosoir ? Oui. Je le porte avec toi. Tu as bien invité. Je suis contente. La joie est là, près des fraisiers. Ils marchent vers la maison, sans se presser. Tu as de la terre aux genoux ? Un peu. C'est tiède. On va laver les mains. Le soleil est encore plus bas.</t>
+          <t>Mila veut poser le bout dans le seau. Le bois est mouillé, un peu sombre. Il la garde ! Mila pousse trop vite, tout de suite. La fraise est trop molle. Elle s'écrase ! Le jus file entre les lattes du seau. Il part ! Un oiseau se pose sur la brouette. Il penche la tête vers le jus. Il veut ma fraise ! Mila avance les mains, trop vite. Puis elle s'arrête net. Mila refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Elle observe la fraise, un instant. Elle écoute le jardin, près du fer. Sur le fer, un éclat de brouette luit. Là, sur le fer. L'oiseau picore la goutte de l'arrosoir. La goutte tombe dans l'herbe. Il a l'eau. On tient le bout ? Oui, papa. Mila lève la fraise hors du seau. Le bout est chaud, un peu plat. Poumf. Il reste sucré, Mila ? Oui, maman. L'oiseau est parti vers le rang. Il a la goutte. Toi, tu as le bout. On le goûte ici ? Oui, près du fer. Mila croque le dernier bout, sans se presser. Il est tiède. Tes genoux sont au chaud ? Un peu, maman. Le jus laisse une trace sur le fer. Il allume le point. Tu vois le point, Mila ? Oui, papa.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Mila se relève. La terre est tiède. On rentre l'arrosoir ? Oui. Je le porte avec toi. Tu as bien invité. Je suis contente. La joie est là, près des fraisiers. Ils marchent vers la maison, sans se presser. Tu as de la terre aux genoux ? Un peu. C'est tiède. On va laver les mains. Le soleil est encore plus bas.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Mila veut poser le bout dans le seau. Le bois est mouillé, un peu sombre. Il la garde ! Mila pousse trop vite, tout de suite. La fraise est trop molle. Elle s'écrase ! Le jus file entre les lattes du seau. Il part ! Un oiseau se pose sur la brouette. Il penche la tête vers le jus. Il veut ma fraise ! Mila avance les mains, trop vite. Puis elle s'arrête net. Mila refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Elle observe la fraise, un instant. Elle écoute le jardin, près du fer. Sur le fer, un &lt;emphasis level="moderate"&gt;éclat de brouette&lt;/emphasis&gt; luit. Là, sur le fer. L'oiseau picore la goutte de l'arrosoir. La goutte tombe dans l'herbe. Il a l'eau. On tient le bout ? Oui, papa. Mila lève la fraise hors du seau. Le bout est chaud, un peu plat. Poumf. Il reste sucré, Mila ? Oui, maman. L'oiseau est parti vers le rang. Il a la goutte. Toi, tu as le bout. On le goûte ici ? Oui, près du fer. Mila croque le dernier bout, sans se presser. Il est tiède. Tes genoux sont au chaud ? Un peu, maman. Le jus laisse une trace sur le fer. Il allume le point. Tu vois le point, Mila ? Oui, papa.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Émeline essuie ses doigts. La terre est tiède. Maman lui prend la &lt;emphasis&gt;main&lt;/emphasis&gt;. [pause]</t>
+          <t>Mila veut poser le bout dans le seau. Le bois est mouillé, un peu sombre. Il la garde ! Mila pousse trop vite, tout de suite. La fraise est trop molle. Elle s'écrase ! Le jus file entre les lattes du seau. Il part ! Un oiseau se pose sur la brouette. Il penche la tête vers le jus. Il veut ma fraise ! Mila avance les mains, trop vite. Puis elle s'arrête net. Mila refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Elle observe la fraise, un instant. Elle écoute le jardin, près du fer. Sur le fer, un &lt;emphasis&gt;éclat de brouette&lt;/emphasis&gt; luit. Là, sur le fer. L'oiseau picore la goutte de l'arrosoir. La goutte tombe dans l'herbe. Il a l'eau. On tient le bout ? Oui, papa. Mila lève la fraise hors du seau. Le bout est chaud, un peu plat. Poumf. Il reste sucré, Mila ? Oui, maman. L'oiseau est parti vers le rang. Il a la goutte. Toi, tu as le bout. On le goûte ici ? Oui, près du fer. Mila croque le dernier bout, sans se presser. Il est tiède. Tes genoux sont au chaud ? Un peu, maman. Le jus laisse une trace sur le fer. Il allume le point. Tu vois le point, Mila ? Oui, papa. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1812,7 +1878,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>132</v>
+        <v>146</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1820,10 +1886,10 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.18</v>
+        <v>1.1</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1846,30 +1912,30 @@
       </c>
       <c r="AH5" s="2" t="inlineStr">
         <is>
-          <t>main</t>
+          <t>éclat de brouette</t>
         </is>
       </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>250</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1878,10 +1944,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1892,20 +1958,61 @@
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=oiseau_jus_fraise_molle_elle_refuse_de_foncer; tempo=vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Mila se relève. La terre est tiède.
-maman|On rentre l'arrosoir ?
-enfant-f|Oui. Je le porte avec toi.
-papa|Tu as bien invité.
-enfant-f|Je suis contente.
-maman|La joie est là, près des fraisiers.
-narrateur|Ils marchent vers la maison, sans se presser.
-papa|Tu as de la terre aux genoux ?
-enfant-f|Un peu. C'est tiède.
-maman|On va laver les mains.
-narrateur|Le soleil est encore plus bas.</t>
+          <t>narrateur|Mila veut poser le bout dans le seau.
+narrateur|Le bois est mouillé, un peu sombre.
+enfant-f|Il la garde !
+narrateur|Mila pousse trop vite, tout de suite.
+narrateur|La fraise est trop molle.
+enfant-f|Elle s'écrase !
+narrateur|Le jus file entre les lattes du seau.
+enfant-f|Il part !
+narrateur|Un oiseau se pose sur la brouette.
+narrateur|Il penche la tête vers le jus.
+enfant-f|Il veut ma fraise !
+narrateur|Mila avance les mains, trop vite.
+narrateur|Puis elle s'arrête net.
+narrateur|Mila refuse de foncer, cette fois.
+narrateur|Ses mains se ferment, puis s'ouvrent.
+narrateur|Personne ne dit la suite.
+narrateur|Elle observe la fraise, un instant.
+narrateur|Elle écoute le jardin, près du fer.
+narrateur|Sur le fer, un éclat de brouette luit.
+enfant-f|Là, sur le fer.
+narrateur|L'oiseau picore la goutte de l'arrosoir.
+narrateur|La goutte tombe dans l'herbe.
+enfant-f|Il a l'eau.
+papa|On tient le bout ?
+enfant-f|Oui, papa.
+narrateur|Mila lève la fraise hors du seau.
+narrateur|Le bout est chaud, un peu plat.
+enfant-f|Poumf.
+maman|Il reste sucré, Mila ?
+enfant-f|Oui, maman.
+papa|L'oiseau est parti vers le rang.
+enfant-f|Il a la goutte.
+maman|Toi, tu as le bout.
+papa|On le goûte ici ?
+enfant-f|Oui, près du fer.
+narrateur|Mila croque le dernier bout, sans se presser.
+enfant-f|Il est tiède.
+maman|Tes genoux sont au chaud ?
+enfant-f|Un peu, maman.
+narrateur|Le jus laisse une trace sur le fer.
+enfant-f|Il allume le point.
+papa|Tu vois le point, Mila ?
+enfant-f|Oui, papa.</t>
+        </is>
+      </c>
+      <c r="AX5" t="inlineStr">
+        <is>
+          <t>oiseau</t>
         </is>
       </c>
     </row>
@@ -1932,17 +2039,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>J'ai dit : je suis contente. On a partagé la fraise. Bravo, Mila.</t>
+          <t>Ils restent près de la brouette. Maman essuie un peu de jus. On a goûté, papa. Tu l'as vue, toi ? Oui, sous la feuille. On est bien, ici. Mila tapote le fer du doigt. Il a une trace de fraise. Tu la vois, la trace ? Oui, maman. La goutte est tombée, Mila. Oui, dans l'herbe. Ça sent la terre, un peu tiède. Et le bois, maman. Oui, dans l'air. Le jardin est calme, Mila ? Oui, papa. L'arrosoir reste contre la brouette. Un éclat de brouette tient sur le fer.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>J'ai dit : je suis contente. On a partagé la fraise. Bravo, Mila.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils restent près de la brouette. Maman essuie un peu de jus. On a goûté, papa. Tu l'as vue, toi ? Oui, sous la feuille. On est bien, ici. Mila tapote le fer du doigt. Il a une trace de fraise. Tu la vois, la trace ? Oui, maman. La goutte est tombée, Mila. Oui, dans l'herbe. Ça sent la terre, un peu tiède. Et le bois, maman. Oui, dans l'air. Le jardin est calme, Mila ? Oui, papa. L'arrosoir reste contre la brouette. Un &lt;emphasis level="moderate"&gt;éclat de brouette&lt;/emphasis&gt; tient sur le fer.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils restent près de la brouette. Maman essuie un peu de jus. On a goûté, papa. Tu l'as vue, toi ? Oui, sous la feuille. On est bien, ici. Mila tapote le fer du doigt. Il a une trace de fraise. Tu la vois, la trace ? Oui, maman. La goutte est tombée, Mila. Oui, dans l'herbe. Ça sent la terre, un peu tiède. Et le bois, maman. Oui, dans l'air. Le jardin est calme, Mila ? Oui, papa. L'arrosoir reste contre la brouette. Un &lt;emphasis&gt;éclat de brouette&lt;/emphasis&gt; tient sur le fer.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -1989,7 +2096,7 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
@@ -1997,10 +2104,10 @@
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.26</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2009,12 +2116,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2023,17 +2130,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de brouette</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2042,11 +2153,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2055,26 +2166,46 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse_et_fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_sur_le_fer; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>enfant-f|J'ai dit : je suis contente.
-enfant-f|On a partagé la fraise.
-papa|Bravo, Mila.</t>
+          <t>narrateur|Ils restent près de la brouette.
+narrateur|Maman essuie un peu de jus.
+enfant-f|On a goûté, papa.
+papa|Tu l'as vue, toi ?
+enfant-f|Oui, sous la feuille.
+maman|On est bien, ici.
+narrateur|Mila tapote le fer du doigt.
+enfant-f|Il a une trace de fraise.
+maman|Tu la vois, la trace ?
+enfant-f|Oui, maman.
+papa|La goutte est tombée, Mila.
+enfant-f|Oui, dans l'herbe.
+narrateur|Ça sent la terre, un peu tiède.
+enfant-f|Et le bois, maman.
+maman|Oui, dans l'air.
+papa|Le jardin est calme, Mila ?
+enfant-f|Oui, papa.
+narrateur|L'arrosoir reste contre la brouette.
+narrateur|Un éclat de brouette tient sur le fer.</t>
         </is>
       </c>
     </row>
@@ -2095,7 +2226,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A9"/>
+  <dimension ref="A1:A10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2159,6 +2290,13 @@
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>